<commit_message>
update vocabolari controllati education-level e education-programme
revisione sintassi topConcept ed eliminazione campi vuoti (note)
</commit_message>
<xml_diff>
--- a/assets/controlled-vocabularies/education-and-labour/education-and-training/education-level/education-level.xlsx
+++ b/assets/controlled-vocabularies/education-and-labour/education-and-training/education-level/education-level.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\pc.istat.it\xendesktop\DaaS\vincenzo.piscitelli\Desktop\VOC. TITOLI DI STUDIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E0799E-7F9D-42E3-B38F-AF1CA268156E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29809984-3792-48DC-8C11-DCC0B7855C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="392">
   <si>
     <t>LIVELLO</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>ALT_LAB_EN</t>
-  </si>
-  <si>
-    <t>NOTE</t>
   </si>
   <si>
     <t>ISCED-A</t>
@@ -1835,10 +1832,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M70"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1875,380 +1872,377 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>22</v>
       </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>28</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>29</v>
       </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
         <v>39</v>
       </c>
-      <c r="F6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>40</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>41</v>
       </c>
-      <c r="J6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="1">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
         <v>43</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>44</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>45</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>46</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>47</v>
       </c>
-      <c r="I7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="1">
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>51</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>52</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>53</v>
       </c>
-      <c r="I8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="1">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
         <v>55</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>56</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="F9" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>58</v>
       </c>
-      <c r="I9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="1">
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" t="s">
         <v>60</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>64</v>
       </c>
-      <c r="J10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="1">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
         <v>66</v>
       </c>
-      <c r="H11" t="s">
-        <v>67</v>
-      </c>
       <c r="I11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="1">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>69</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>70</v>
       </c>
-      <c r="I12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" s="1">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
         <v>72</v>
       </c>
-      <c r="E13" t="s">
+      <c r="H13" t="s">
         <v>73</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>74</v>
       </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="1">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
         <v>76</v>
       </c>
-      <c r="E14" t="s">
+      <c r="H14" t="s">
         <v>77</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="I14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="1">
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" t="s">
         <v>80</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>81</v>
       </c>
-      <c r="E15" t="s">
+      <c r="H15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>83</v>
       </c>
-      <c r="I15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" s="1">
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
         <v>85</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>86</v>
       </c>
-      <c r="E16" t="s">
+      <c r="H16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>88</v>
-      </c>
-      <c r="I16" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -2256,22 +2250,22 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" t="s">
         <v>90</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>91</v>
       </c>
-      <c r="E17" t="s">
+      <c r="H17" t="s">
         <v>92</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>93</v>
-      </c>
-      <c r="I17" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -2279,22 +2273,22 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
         <v>95</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>96</v>
       </c>
-      <c r="E18" t="s">
+      <c r="H18" t="s">
         <v>97</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>98</v>
-      </c>
-      <c r="I18" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -2302,25 +2296,25 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="s">
         <v>100</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>101</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+      <c r="H19" t="s">
         <v>102</v>
       </c>
-      <c r="F19" t="s">
-        <v>95</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>103</v>
-      </c>
-      <c r="I19" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -2328,28 +2322,28 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
         <v>105</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>106</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" t="s">
         <v>107</v>
       </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>108</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>109</v>
-      </c>
-      <c r="J20" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2357,28 +2351,28 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21" t="s">
         <v>111</v>
-      </c>
-      <c r="D21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21" t="s">
-        <v>22</v>
-      </c>
-      <c r="I21" t="s">
-        <v>23</v>
-      </c>
-      <c r="J21" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2386,25 +2380,25 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
         <v>113</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>114</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>115</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
+        <v>24</v>
+      </c>
+      <c r="H22" t="s">
         <v>116</v>
       </c>
-      <c r="F22" t="s">
-        <v>25</v>
-      </c>
-      <c r="H22" t="s">
-        <v>117</v>
-      </c>
       <c r="I22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2412,28 +2406,28 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" t="s">
         <v>118</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>119</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" t="s">
         <v>120</v>
       </c>
-      <c r="F23" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
+        <v>116</v>
+      </c>
+      <c r="I23" t="s">
         <v>121</v>
-      </c>
-      <c r="H23" t="s">
-        <v>117</v>
-      </c>
-      <c r="I23" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2441,25 +2435,25 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" t="s">
         <v>123</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>124</v>
       </c>
-      <c r="E24" t="s">
-        <v>125</v>
-      </c>
       <c r="F24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2467,28 +2461,28 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" t="s">
         <v>126</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>127</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
+        <v>30</v>
+      </c>
+      <c r="G25" t="s">
         <v>128</v>
       </c>
-      <c r="F25" t="s">
-        <v>31</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>129</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>130</v>
-      </c>
-      <c r="I25" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2496,28 +2490,28 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" t="s">
         <v>132</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>133</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" t="s">
         <v>134</v>
       </c>
-      <c r="F26" t="s">
-        <v>31</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>135</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>136</v>
-      </c>
-      <c r="I26" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2525,31 +2519,31 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C27" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" t="s">
         <v>138</v>
       </c>
-      <c r="D27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
         <v>139</v>
       </c>
-      <c r="F27" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" t="s">
-        <v>140</v>
-      </c>
       <c r="H27" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" t="s">
         <v>40</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>41</v>
-      </c>
-      <c r="J27" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2557,31 +2551,31 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C28" t="s">
+        <v>140</v>
+      </c>
+      <c r="D28" t="s">
         <v>141</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>142</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" t="s">
         <v>143</v>
       </c>
-      <c r="F28" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>144</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>145</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>146</v>
-      </c>
-      <c r="J28" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -2589,31 +2583,31 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C29" t="s">
+        <v>147</v>
+      </c>
+      <c r="D29" t="s">
         <v>148</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>149</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" t="s">
         <v>150</v>
       </c>
-      <c r="F29" t="s">
-        <v>43</v>
-      </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>151</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>152</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>153</v>
-      </c>
-      <c r="J29" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -2621,31 +2615,31 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
+        <v>154</v>
+      </c>
+      <c r="D30" t="s">
         <v>155</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>156</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
+        <v>48</v>
+      </c>
+      <c r="G30" t="s">
         <v>157</v>
       </c>
-      <c r="F30" t="s">
-        <v>49</v>
-      </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>158</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>159</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>160</v>
-      </c>
-      <c r="J30" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -2653,28 +2647,28 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C31" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" t="s">
         <v>162</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>163</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" t="s">
         <v>164</v>
       </c>
-      <c r="F31" t="s">
-        <v>49</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>165</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>166</v>
-      </c>
-      <c r="I31" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -2682,31 +2676,31 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C32" t="s">
+        <v>167</v>
+      </c>
+      <c r="D32" t="s">
         <v>168</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>169</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
+        <v>48</v>
+      </c>
+      <c r="G32" t="s">
         <v>170</v>
       </c>
-      <c r="F32" t="s">
-        <v>49</v>
-      </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>171</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>172</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>173</v>
-      </c>
-      <c r="J32" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -2714,31 +2708,31 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
+        <v>174</v>
+      </c>
+      <c r="D33" t="s">
         <v>175</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>176</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" t="s">
         <v>177</v>
       </c>
-      <c r="F33" t="s">
-        <v>55</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>178</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>179</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>180</v>
-      </c>
-      <c r="J33" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -2746,28 +2740,28 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C34" t="s">
+        <v>181</v>
+      </c>
+      <c r="D34" t="s">
         <v>182</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>183</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" t="s">
         <v>184</v>
       </c>
-      <c r="F34" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>185</v>
       </c>
-      <c r="H34" t="s">
-        <v>186</v>
-      </c>
       <c r="I34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -2775,25 +2769,25 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C35" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" t="s">
         <v>187</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>188</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
+        <v>79</v>
+      </c>
+      <c r="H35" t="s">
         <v>189</v>
       </c>
-      <c r="F35" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>190</v>
-      </c>
-      <c r="I35" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -2801,25 +2795,25 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s">
+        <v>191</v>
+      </c>
+      <c r="D36" t="s">
         <v>192</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>193</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
+        <v>84</v>
+      </c>
+      <c r="H36" t="s">
         <v>194</v>
       </c>
-      <c r="F36" t="s">
-        <v>85</v>
-      </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>195</v>
-      </c>
-      <c r="I36" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -2827,25 +2821,25 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
+        <v>196</v>
+      </c>
+      <c r="D37" t="s">
         <v>197</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>198</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H37" t="s">
         <v>199</v>
       </c>
-      <c r="F37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>200</v>
-      </c>
-      <c r="I37" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2853,28 +2847,28 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C38" t="s">
+        <v>201</v>
+      </c>
+      <c r="D38" t="s">
         <v>202</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>203</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
+        <v>89</v>
+      </c>
+      <c r="H38" t="s">
         <v>204</v>
       </c>
-      <c r="F38" t="s">
-        <v>90</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
         <v>205</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>206</v>
-      </c>
-      <c r="J38" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2882,28 +2876,28 @@
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
+        <v>207</v>
+      </c>
+      <c r="D39" t="s">
         <v>208</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>209</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
+        <v>89</v>
+      </c>
+      <c r="H39" t="s">
         <v>210</v>
       </c>
-      <c r="F39" t="s">
-        <v>90</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="I39" t="s">
         <v>211</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>212</v>
-      </c>
-      <c r="J39" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2911,25 +2905,25 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C40" t="s">
+        <v>213</v>
+      </c>
+      <c r="D40" t="s">
         <v>214</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>215</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
+        <v>89</v>
+      </c>
+      <c r="H40" t="s">
         <v>216</v>
       </c>
-      <c r="F40" t="s">
-        <v>90</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>217</v>
-      </c>
-      <c r="I40" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2937,28 +2931,28 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C41" t="s">
+        <v>218</v>
+      </c>
+      <c r="D41" t="s">
         <v>219</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>220</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
+        <v>89</v>
+      </c>
+      <c r="H41" t="s">
         <v>221</v>
       </c>
-      <c r="F41" t="s">
-        <v>90</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>222</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>223</v>
-      </c>
-      <c r="J41" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -2966,25 +2960,25 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C42" t="s">
+        <v>224</v>
+      </c>
+      <c r="D42" t="s">
         <v>225</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>226</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>94</v>
+      </c>
+      <c r="H42" t="s">
         <v>227</v>
       </c>
-      <c r="F42" t="s">
-        <v>95</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>228</v>
-      </c>
-      <c r="I42" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -2992,25 +2986,25 @@
         <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43" t="s">
+        <v>229</v>
+      </c>
+      <c r="D43" t="s">
         <v>230</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>231</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
+        <v>94</v>
+      </c>
+      <c r="H43" t="s">
         <v>232</v>
       </c>
-      <c r="F43" t="s">
-        <v>95</v>
-      </c>
-      <c r="H43" t="s">
+      <c r="I43" t="s">
         <v>233</v>
-      </c>
-      <c r="I43" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3018,28 +3012,28 @@
         <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C44" t="s">
+        <v>234</v>
+      </c>
+      <c r="D44" t="s">
         <v>235</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>236</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
+        <v>94</v>
+      </c>
+      <c r="H44" t="s">
         <v>237</v>
       </c>
-      <c r="F44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>238</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>239</v>
-      </c>
-      <c r="J44" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -3047,31 +3041,31 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C45" t="s">
+        <v>240</v>
+      </c>
+      <c r="D45" t="s">
         <v>241</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>242</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
+        <v>224</v>
+      </c>
+      <c r="G45" t="s">
         <v>243</v>
       </c>
-      <c r="F45" t="s">
-        <v>225</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>244</v>
       </c>
-      <c r="H45" t="s">
+      <c r="I45" t="s">
         <v>245</v>
       </c>
-      <c r="I45" t="s">
+      <c r="J45" t="s">
         <v>246</v>
-      </c>
-      <c r="J45" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -3079,31 +3073,31 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C46" t="s">
+        <v>247</v>
+      </c>
+      <c r="D46" t="s">
         <v>248</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>249</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
+        <v>224</v>
+      </c>
+      <c r="G46" t="s">
         <v>250</v>
       </c>
-      <c r="F46" t="s">
-        <v>225</v>
-      </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>251</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>252</v>
       </c>
-      <c r="I46" t="s">
+      <c r="J46" t="s">
         <v>253</v>
-      </c>
-      <c r="J46" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -3111,31 +3105,31 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C47" t="s">
+        <v>254</v>
+      </c>
+      <c r="D47" t="s">
         <v>255</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>256</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
+        <v>224</v>
+      </c>
+      <c r="G47" t="s">
         <v>257</v>
       </c>
-      <c r="F47" t="s">
-        <v>225</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>258</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
         <v>259</v>
       </c>
-      <c r="I47" t="s">
+      <c r="J47" t="s">
         <v>260</v>
-      </c>
-      <c r="J47" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -3143,31 +3137,31 @@
         <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D48" t="s">
         <v>262</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>263</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>229</v>
+      </c>
+      <c r="G48" t="s">
         <v>264</v>
       </c>
-      <c r="F48" t="s">
-        <v>230</v>
-      </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>265</v>
       </c>
-      <c r="H48" t="s">
+      <c r="I48" t="s">
         <v>266</v>
       </c>
-      <c r="I48" t="s">
+      <c r="J48" t="s">
         <v>267</v>
-      </c>
-      <c r="J48" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -3175,31 +3169,31 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C49" t="s">
+        <v>268</v>
+      </c>
+      <c r="D49" t="s">
         <v>269</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>270</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
+        <v>229</v>
+      </c>
+      <c r="G49" t="s">
         <v>271</v>
       </c>
-      <c r="F49" t="s">
-        <v>230</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>272</v>
       </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>273</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" t="s">
         <v>274</v>
-      </c>
-      <c r="J49" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -3207,31 +3201,31 @@
         <v>3</v>
       </c>
       <c r="B50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
+        <v>275</v>
+      </c>
+      <c r="D50" t="s">
         <v>276</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>277</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
+        <v>229</v>
+      </c>
+      <c r="G50" t="s">
         <v>278</v>
       </c>
-      <c r="F50" t="s">
-        <v>230</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>279</v>
       </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
         <v>280</v>
       </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>281</v>
-      </c>
-      <c r="J50" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -3239,31 +3233,31 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" t="s">
+        <v>282</v>
+      </c>
+      <c r="D51" t="s">
         <v>283</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>284</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
+        <v>234</v>
+      </c>
+      <c r="G51" t="s">
         <v>285</v>
       </c>
-      <c r="F51" t="s">
-        <v>235</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>286</v>
       </c>
-      <c r="H51" t="s">
+      <c r="I51" t="s">
         <v>287</v>
       </c>
-      <c r="I51" t="s">
-        <v>288</v>
-      </c>
       <c r="J51" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -3271,31 +3265,31 @@
         <v>3</v>
       </c>
       <c r="B52" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C52" t="s">
+        <v>288</v>
+      </c>
+      <c r="D52" t="s">
         <v>289</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>290</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>234</v>
+      </c>
+      <c r="G52" t="s">
         <v>291</v>
       </c>
-      <c r="F52" t="s">
-        <v>235</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>292</v>
       </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>293</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>294</v>
-      </c>
-      <c r="J52" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -3303,31 +3297,31 @@
         <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C53" t="s">
+        <v>295</v>
+      </c>
+      <c r="D53" t="s">
+        <v>100</v>
+      </c>
+      <c r="E53" t="s">
+        <v>101</v>
+      </c>
+      <c r="F53" t="s">
+        <v>99</v>
+      </c>
+      <c r="G53" t="s">
         <v>296</v>
       </c>
-      <c r="D53" t="s">
-        <v>101</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="H53" t="s">
         <v>102</v>
       </c>
-      <c r="F53" t="s">
-        <v>100</v>
-      </c>
-      <c r="G53" t="s">
+      <c r="I53" t="s">
+        <v>103</v>
+      </c>
+      <c r="J53" t="s">
         <v>297</v>
-      </c>
-      <c r="H53" t="s">
-        <v>103</v>
-      </c>
-      <c r="I53" t="s">
-        <v>104</v>
-      </c>
-      <c r="J53" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -3335,31 +3329,31 @@
         <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C54" t="s">
+        <v>298</v>
+      </c>
+      <c r="D54" t="s">
         <v>299</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>300</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
+        <v>104</v>
+      </c>
+      <c r="G54" t="s">
         <v>301</v>
       </c>
-      <c r="F54" t="s">
-        <v>105</v>
-      </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>302</v>
       </c>
-      <c r="H54" t="s">
+      <c r="I54" t="s">
         <v>303</v>
       </c>
-      <c r="I54" t="s">
+      <c r="J54" t="s">
         <v>304</v>
-      </c>
-      <c r="J54" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -3367,31 +3361,31 @@
         <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C55" t="s">
+        <v>305</v>
+      </c>
+      <c r="D55" t="s">
         <v>306</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>307</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
+        <v>59</v>
+      </c>
+      <c r="G55" t="s">
         <v>308</v>
       </c>
-      <c r="F55" t="s">
-        <v>60</v>
-      </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>309</v>
       </c>
-      <c r="H55" t="s">
+      <c r="I55" t="s">
         <v>310</v>
       </c>
-      <c r="I55" t="s">
+      <c r="J55" t="s">
         <v>311</v>
-      </c>
-      <c r="J55" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -3399,31 +3393,31 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C56" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" t="s">
         <v>313</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>314</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
+        <v>59</v>
+      </c>
+      <c r="G56" t="s">
         <v>315</v>
       </c>
-      <c r="F56" t="s">
-        <v>60</v>
-      </c>
-      <c r="G56" t="s">
+      <c r="H56" t="s">
         <v>316</v>
       </c>
-      <c r="H56" t="s">
+      <c r="I56" t="s">
         <v>317</v>
       </c>
-      <c r="I56" t="s">
+      <c r="J56" t="s">
         <v>318</v>
-      </c>
-      <c r="J56" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -3431,28 +3425,28 @@
         <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C57" t="s">
+        <v>319</v>
+      </c>
+      <c r="D57" t="s">
         <v>320</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>321</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
+        <v>186</v>
+      </c>
+      <c r="G57" t="s">
         <v>322</v>
       </c>
-      <c r="F57" t="s">
-        <v>187</v>
-      </c>
-      <c r="G57" t="s">
+      <c r="H57" t="s">
         <v>323</v>
       </c>
-      <c r="H57" t="s">
+      <c r="I57" t="s">
         <v>324</v>
-      </c>
-      <c r="I57" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -3460,31 +3454,31 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C58" t="s">
+        <v>325</v>
+      </c>
+      <c r="D58" t="s">
         <v>326</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>327</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
+        <v>186</v>
+      </c>
+      <c r="G58" t="s">
         <v>328</v>
       </c>
-      <c r="F58" t="s">
-        <v>187</v>
-      </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>329</v>
       </c>
-      <c r="H58" t="s">
+      <c r="I58" t="s">
         <v>330</v>
       </c>
-      <c r="I58" t="s">
+      <c r="J58" t="s">
         <v>331</v>
-      </c>
-      <c r="J58" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -3492,31 +3486,31 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C59" t="s">
+        <v>332</v>
+      </c>
+      <c r="D59" t="s">
         <v>333</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>334</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
+        <v>191</v>
+      </c>
+      <c r="G59" t="s">
         <v>335</v>
       </c>
-      <c r="F59" t="s">
-        <v>192</v>
-      </c>
-      <c r="G59" t="s">
+      <c r="H59" t="s">
         <v>336</v>
       </c>
-      <c r="H59" t="s">
+      <c r="I59" t="s">
         <v>337</v>
       </c>
-      <c r="I59" t="s">
+      <c r="J59" t="s">
         <v>338</v>
-      </c>
-      <c r="J59" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -3524,31 +3518,31 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C60" t="s">
+        <v>339</v>
+      </c>
+      <c r="D60" t="s">
         <v>340</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>341</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
+        <v>191</v>
+      </c>
+      <c r="G60" t="s">
         <v>342</v>
       </c>
-      <c r="F60" t="s">
-        <v>192</v>
-      </c>
-      <c r="G60" t="s">
+      <c r="H60" t="s">
         <v>343</v>
       </c>
-      <c r="H60" t="s">
+      <c r="I60" t="s">
         <v>344</v>
       </c>
-      <c r="I60" t="s">
+      <c r="J60" t="s">
         <v>345</v>
-      </c>
-      <c r="J60" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -3556,28 +3550,28 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C61" t="s">
+        <v>346</v>
+      </c>
+      <c r="D61" t="s">
+        <v>197</v>
+      </c>
+      <c r="E61" t="s">
+        <v>198</v>
+      </c>
+      <c r="F61" t="s">
+        <v>196</v>
+      </c>
+      <c r="G61" t="s">
         <v>347</v>
       </c>
-      <c r="D61" t="s">
-        <v>198</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="H61" t="s">
         <v>199</v>
       </c>
-      <c r="F61" t="s">
-        <v>197</v>
-      </c>
-      <c r="G61" t="s">
-        <v>348</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="I61" t="s">
         <v>200</v>
-      </c>
-      <c r="I61" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -3585,31 +3579,31 @@
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C62" t="s">
+        <v>348</v>
+      </c>
+      <c r="D62" t="s">
+        <v>202</v>
+      </c>
+      <c r="E62" t="s">
+        <v>203</v>
+      </c>
+      <c r="F62" t="s">
+        <v>201</v>
+      </c>
+      <c r="G62" t="s">
         <v>349</v>
       </c>
-      <c r="D62" t="s">
-        <v>203</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="H62" t="s">
         <v>204</v>
       </c>
-      <c r="F62" t="s">
-        <v>202</v>
-      </c>
-      <c r="G62" t="s">
+      <c r="I62" t="s">
+        <v>205</v>
+      </c>
+      <c r="J62" t="s">
         <v>350</v>
-      </c>
-      <c r="H62" t="s">
-        <v>205</v>
-      </c>
-      <c r="I62" t="s">
-        <v>206</v>
-      </c>
-      <c r="J62" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -3617,31 +3611,31 @@
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C63" t="s">
+        <v>351</v>
+      </c>
+      <c r="D63" t="s">
+        <v>208</v>
+      </c>
+      <c r="E63" t="s">
         <v>352</v>
       </c>
-      <c r="D63" t="s">
-        <v>209</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
+        <v>207</v>
+      </c>
+      <c r="G63" t="s">
         <v>353</v>
       </c>
-      <c r="F63" t="s">
-        <v>208</v>
-      </c>
-      <c r="G63" t="s">
-        <v>354</v>
-      </c>
       <c r="H63" t="s">
+        <v>210</v>
+      </c>
+      <c r="I63" t="s">
         <v>211</v>
       </c>
-      <c r="I63" t="s">
+      <c r="J63" t="s">
         <v>212</v>
-      </c>
-      <c r="J63" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -3649,28 +3643,28 @@
         <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C64" t="s">
+        <v>354</v>
+      </c>
+      <c r="D64" t="s">
+        <v>214</v>
+      </c>
+      <c r="E64" t="s">
+        <v>215</v>
+      </c>
+      <c r="F64" t="s">
+        <v>213</v>
+      </c>
+      <c r="G64" t="s">
         <v>355</v>
       </c>
-      <c r="D64" t="s">
-        <v>215</v>
-      </c>
-      <c r="E64" t="s">
+      <c r="H64" t="s">
         <v>216</v>
       </c>
-      <c r="F64" t="s">
-        <v>214</v>
-      </c>
-      <c r="G64" t="s">
-        <v>356</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>217</v>
-      </c>
-      <c r="I64" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -3678,31 +3672,31 @@
         <v>3</v>
       </c>
       <c r="B65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C65" t="s">
+        <v>356</v>
+      </c>
+      <c r="D65" t="s">
         <v>357</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>358</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
+        <v>218</v>
+      </c>
+      <c r="G65" t="s">
         <v>359</v>
       </c>
-      <c r="F65" t="s">
-        <v>219</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>360</v>
       </c>
-      <c r="H65" t="s">
+      <c r="I65" t="s">
         <v>361</v>
       </c>
-      <c r="I65" t="s">
-        <v>362</v>
-      </c>
       <c r="J65" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -3710,31 +3704,31 @@
         <v>3</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C66" t="s">
+        <v>362</v>
+      </c>
+      <c r="D66" t="s">
         <v>363</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>364</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
+        <v>218</v>
+      </c>
+      <c r="G66" t="s">
         <v>365</v>
       </c>
-      <c r="F66" t="s">
-        <v>219</v>
-      </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>366</v>
       </c>
-      <c r="H66" t="s">
+      <c r="I66" t="s">
         <v>367</v>
       </c>
-      <c r="I66" t="s">
+      <c r="J66" t="s">
         <v>368</v>
-      </c>
-      <c r="J66" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -3742,31 +3736,31 @@
         <v>3</v>
       </c>
       <c r="B67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C67" t="s">
+        <v>369</v>
+      </c>
+      <c r="D67" t="s">
         <v>370</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>371</v>
       </c>
-      <c r="E67" t="s">
+      <c r="F67" t="s">
+        <v>104</v>
+      </c>
+      <c r="G67" t="s">
         <v>372</v>
       </c>
-      <c r="F67" t="s">
-        <v>105</v>
-      </c>
-      <c r="G67" t="s">
+      <c r="H67" t="s">
         <v>373</v>
       </c>
-      <c r="H67" t="s">
+      <c r="I67" t="s">
         <v>374</v>
       </c>
-      <c r="I67" t="s">
-        <v>375</v>
-      </c>
       <c r="J67" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -3774,28 +3768,28 @@
         <v>3</v>
       </c>
       <c r="B68" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C68" t="s">
+        <v>375</v>
+      </c>
+      <c r="D68" t="s">
         <v>376</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>377</v>
       </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" t="s">
         <v>378</v>
       </c>
-      <c r="F68" t="s">
-        <v>111</v>
-      </c>
-      <c r="G68" t="s">
+      <c r="H68" t="s">
         <v>379</v>
       </c>
-      <c r="H68" t="s">
-        <v>380</v>
-      </c>
       <c r="I68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -3803,28 +3797,28 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C69" t="s">
+        <v>380</v>
+      </c>
+      <c r="D69" t="s">
         <v>381</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>382</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>383</v>
       </c>
-      <c r="F69" t="s">
+      <c r="G69" t="s">
         <v>384</v>
       </c>
-      <c r="G69" t="s">
+      <c r="H69" t="s">
         <v>385</v>
       </c>
-      <c r="H69" t="s">
-        <v>386</v>
-      </c>
       <c r="I69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -3832,28 +3826,28 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C70" t="s">
+        <v>386</v>
+      </c>
+      <c r="D70" t="s">
         <v>387</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>388</v>
       </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>389</v>
       </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>390</v>
       </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>391</v>
       </c>
-      <c r="H70" t="s">
-        <v>392</v>
-      </c>
       <c r="I70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update vocabolari controllati education-level e education-programme (#61)
* creazione vocabolari controllati titoli e programmi

creazione vocabolari controllati titoli e programmi di istruzione (senza distributions)

* update

* update vocabolari controllati titoli e percorsi di studio

aggiornamento metadati vocabolari controllati titoli e percorsi di studio

* update vocabolari education-level e programme

inserito prefix per migliorare visualizzazione su lodview

* update vocabolari controllati education-level e education-programme

revisione sintassi topConcept ed eliminazione campi vuoti (note)
</commit_message>
<xml_diff>
--- a/assets/controlled-vocabularies/education-and-labour/education-and-training/education-level/education-level.xlsx
+++ b/assets/controlled-vocabularies/education-and-labour/education-and-training/education-level/education-level.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\pc.istat.it\xendesktop\DaaS\vincenzo.piscitelli\Desktop\VOC. TITOLI DI STUDIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E0799E-7F9D-42E3-B38F-AF1CA268156E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29809984-3792-48DC-8C11-DCC0B7855C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="392">
   <si>
     <t>LIVELLO</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>ALT_LAB_EN</t>
-  </si>
-  <si>
-    <t>NOTE</t>
   </si>
   <si>
     <t>ISCED-A</t>
@@ -1835,10 +1832,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M70"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1875,380 +1872,377 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>22</v>
       </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>25</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>27</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>28</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>29</v>
       </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>38</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
         <v>39</v>
       </c>
-      <c r="F6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>40</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>41</v>
       </c>
-      <c r="J6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="1">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" t="s">
         <v>43</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>44</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>45</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>46</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>47</v>
       </c>
-      <c r="I7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="1">
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>51</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>52</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>53</v>
       </c>
-      <c r="I8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="1">
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
         <v>55</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>56</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="F9" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>58</v>
       </c>
-      <c r="I9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="1">
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" t="s">
         <v>60</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" t="s">
         <v>62</v>
       </c>
-      <c r="F10" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>63</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>64</v>
       </c>
-      <c r="J10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="1">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
         <v>66</v>
       </c>
-      <c r="H11" t="s">
-        <v>67</v>
-      </c>
       <c r="I11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="1">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
         <v>69</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>70</v>
       </c>
-      <c r="I12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" s="1">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
         <v>72</v>
       </c>
-      <c r="E13" t="s">
+      <c r="H13" t="s">
         <v>73</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>74</v>
       </c>
-      <c r="I13" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="1">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
         <v>76</v>
       </c>
-      <c r="E14" t="s">
+      <c r="H14" t="s">
         <v>77</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="I14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="1">
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" t="s">
         <v>80</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>81</v>
       </c>
-      <c r="E15" t="s">
+      <c r="H15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>83</v>
       </c>
-      <c r="I15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" s="1">
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D16" t="s">
         <v>85</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>86</v>
       </c>
-      <c r="E16" t="s">
+      <c r="H16" t="s">
         <v>87</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>88</v>
-      </c>
-      <c r="I16" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -2256,22 +2250,22 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" t="s">
         <v>90</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>91</v>
       </c>
-      <c r="E17" t="s">
+      <c r="H17" t="s">
         <v>92</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>93</v>
-      </c>
-      <c r="I17" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -2279,22 +2273,22 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" t="s">
         <v>95</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>96</v>
       </c>
-      <c r="E18" t="s">
+      <c r="H18" t="s">
         <v>97</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>98</v>
-      </c>
-      <c r="I18" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -2302,25 +2296,25 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" t="s">
         <v>100</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>101</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+      <c r="H19" t="s">
         <v>102</v>
       </c>
-      <c r="F19" t="s">
-        <v>95</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>103</v>
-      </c>
-      <c r="I19" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -2328,28 +2322,28 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
         <v>105</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>106</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" t="s">
         <v>107</v>
       </c>
-      <c r="F20" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>108</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>109</v>
-      </c>
-      <c r="J20" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -2357,28 +2351,28 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" t="s">
+        <v>21</v>
+      </c>
+      <c r="I21" t="s">
+        <v>22</v>
+      </c>
+      <c r="J21" t="s">
         <v>111</v>
-      </c>
-      <c r="D21" t="s">
-        <v>20</v>
-      </c>
-      <c r="E21" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21" t="s">
-        <v>22</v>
-      </c>
-      <c r="I21" t="s">
-        <v>23</v>
-      </c>
-      <c r="J21" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2386,25 +2380,25 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
         <v>113</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>114</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>115</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
+        <v>24</v>
+      </c>
+      <c r="H22" t="s">
         <v>116</v>
       </c>
-      <c r="F22" t="s">
-        <v>25</v>
-      </c>
-      <c r="H22" t="s">
-        <v>117</v>
-      </c>
       <c r="I22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -2412,28 +2406,28 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" t="s">
         <v>118</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>119</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" t="s">
         <v>120</v>
       </c>
-      <c r="F23" t="s">
-        <v>25</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
+        <v>116</v>
+      </c>
+      <c r="I23" t="s">
         <v>121</v>
-      </c>
-      <c r="H23" t="s">
-        <v>117</v>
-      </c>
-      <c r="I23" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -2441,25 +2435,25 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" t="s">
         <v>123</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>124</v>
       </c>
-      <c r="E24" t="s">
-        <v>125</v>
-      </c>
       <c r="F24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -2467,28 +2461,28 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C25" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" t="s">
         <v>126</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>127</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
+        <v>30</v>
+      </c>
+      <c r="G25" t="s">
         <v>128</v>
       </c>
-      <c r="F25" t="s">
-        <v>31</v>
-      </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>129</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>130</v>
-      </c>
-      <c r="I25" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -2496,28 +2490,28 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" t="s">
         <v>132</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>133</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" t="s">
         <v>134</v>
       </c>
-      <c r="F26" t="s">
-        <v>31</v>
-      </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>135</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>136</v>
-      </c>
-      <c r="I26" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -2525,31 +2519,31 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C27" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" t="s">
         <v>138</v>
       </c>
-      <c r="D27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
+        <v>30</v>
+      </c>
+      <c r="G27" t="s">
         <v>139</v>
       </c>
-      <c r="F27" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" t="s">
-        <v>140</v>
-      </c>
       <c r="H27" t="s">
+        <v>39</v>
+      </c>
+      <c r="I27" t="s">
         <v>40</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>41</v>
-      </c>
-      <c r="J27" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -2557,31 +2551,31 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C28" t="s">
+        <v>140</v>
+      </c>
+      <c r="D28" t="s">
         <v>141</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>142</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" t="s">
         <v>143</v>
       </c>
-      <c r="F28" t="s">
-        <v>43</v>
-      </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>144</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>145</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>146</v>
-      </c>
-      <c r="J28" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -2589,31 +2583,31 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C29" t="s">
+        <v>147</v>
+      </c>
+      <c r="D29" t="s">
         <v>148</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>149</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" t="s">
         <v>150</v>
       </c>
-      <c r="F29" t="s">
-        <v>43</v>
-      </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>151</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>152</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>153</v>
-      </c>
-      <c r="J29" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -2621,31 +2615,31 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
+        <v>154</v>
+      </c>
+      <c r="D30" t="s">
         <v>155</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>156</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
+        <v>48</v>
+      </c>
+      <c r="G30" t="s">
         <v>157</v>
       </c>
-      <c r="F30" t="s">
-        <v>49</v>
-      </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>158</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>159</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>160</v>
-      </c>
-      <c r="J30" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -2653,28 +2647,28 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C31" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" t="s">
         <v>162</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>163</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" t="s">
         <v>164</v>
       </c>
-      <c r="F31" t="s">
-        <v>49</v>
-      </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>165</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>166</v>
-      </c>
-      <c r="I31" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -2682,31 +2676,31 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C32" t="s">
+        <v>167</v>
+      </c>
+      <c r="D32" t="s">
         <v>168</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>169</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
+        <v>48</v>
+      </c>
+      <c r="G32" t="s">
         <v>170</v>
       </c>
-      <c r="F32" t="s">
-        <v>49</v>
-      </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>171</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>172</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>173</v>
-      </c>
-      <c r="J32" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -2714,31 +2708,31 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
+        <v>174</v>
+      </c>
+      <c r="D33" t="s">
         <v>175</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>176</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" t="s">
         <v>177</v>
       </c>
-      <c r="F33" t="s">
-        <v>55</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>178</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>179</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>180</v>
-      </c>
-      <c r="J33" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -2746,28 +2740,28 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C34" t="s">
+        <v>181</v>
+      </c>
+      <c r="D34" t="s">
         <v>182</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>183</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" t="s">
         <v>184</v>
       </c>
-      <c r="F34" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>185</v>
       </c>
-      <c r="H34" t="s">
-        <v>186</v>
-      </c>
       <c r="I34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -2775,25 +2769,25 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C35" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" t="s">
         <v>187</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>188</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
+        <v>79</v>
+      </c>
+      <c r="H35" t="s">
         <v>189</v>
       </c>
-      <c r="F35" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>190</v>
-      </c>
-      <c r="I35" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -2801,25 +2795,25 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s">
+        <v>191</v>
+      </c>
+      <c r="D36" t="s">
         <v>192</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>193</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
+        <v>84</v>
+      </c>
+      <c r="H36" t="s">
         <v>194</v>
       </c>
-      <c r="F36" t="s">
-        <v>85</v>
-      </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>195</v>
-      </c>
-      <c r="I36" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -2827,25 +2821,25 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s">
+        <v>196</v>
+      </c>
+      <c r="D37" t="s">
         <v>197</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>198</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
+        <v>89</v>
+      </c>
+      <c r="H37" t="s">
         <v>199</v>
       </c>
-      <c r="F37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>200</v>
-      </c>
-      <c r="I37" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2853,28 +2847,28 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C38" t="s">
+        <v>201</v>
+      </c>
+      <c r="D38" t="s">
         <v>202</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>203</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
+        <v>89</v>
+      </c>
+      <c r="H38" t="s">
         <v>204</v>
       </c>
-      <c r="F38" t="s">
-        <v>90</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
         <v>205</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>206</v>
-      </c>
-      <c r="J38" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2882,28 +2876,28 @@
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C39" t="s">
+        <v>207</v>
+      </c>
+      <c r="D39" t="s">
         <v>208</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>209</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
+        <v>89</v>
+      </c>
+      <c r="H39" t="s">
         <v>210</v>
       </c>
-      <c r="F39" t="s">
-        <v>90</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="I39" t="s">
         <v>211</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>212</v>
-      </c>
-      <c r="J39" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -2911,25 +2905,25 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C40" t="s">
+        <v>213</v>
+      </c>
+      <c r="D40" t="s">
         <v>214</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>215</v>
       </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
+        <v>89</v>
+      </c>
+      <c r="H40" t="s">
         <v>216</v>
       </c>
-      <c r="F40" t="s">
-        <v>90</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>217</v>
-      </c>
-      <c r="I40" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2937,28 +2931,28 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C41" t="s">
+        <v>218</v>
+      </c>
+      <c r="D41" t="s">
         <v>219</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>220</v>
       </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
+        <v>89</v>
+      </c>
+      <c r="H41" t="s">
         <v>221</v>
       </c>
-      <c r="F41" t="s">
-        <v>90</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>222</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>223</v>
-      </c>
-      <c r="J41" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:10">
@@ -2966,25 +2960,25 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C42" t="s">
+        <v>224</v>
+      </c>
+      <c r="D42" t="s">
         <v>225</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>226</v>
       </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>94</v>
+      </c>
+      <c r="H42" t="s">
         <v>227</v>
       </c>
-      <c r="F42" t="s">
-        <v>95</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>228</v>
-      </c>
-      <c r="I42" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -2992,25 +2986,25 @@
         <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43" t="s">
+        <v>229</v>
+      </c>
+      <c r="D43" t="s">
         <v>230</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>231</v>
       </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
+        <v>94</v>
+      </c>
+      <c r="H43" t="s">
         <v>232</v>
       </c>
-      <c r="F43" t="s">
-        <v>95</v>
-      </c>
-      <c r="H43" t="s">
+      <c r="I43" t="s">
         <v>233</v>
-      </c>
-      <c r="I43" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -3018,28 +3012,28 @@
         <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C44" t="s">
+        <v>234</v>
+      </c>
+      <c r="D44" t="s">
         <v>235</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>236</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
+        <v>94</v>
+      </c>
+      <c r="H44" t="s">
         <v>237</v>
       </c>
-      <c r="F44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>238</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>239</v>
-      </c>
-      <c r="J44" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -3047,31 +3041,31 @@
         <v>3</v>
       </c>
       <c r="B45" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C45" t="s">
+        <v>240</v>
+      </c>
+      <c r="D45" t="s">
         <v>241</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>242</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
+        <v>224</v>
+      </c>
+      <c r="G45" t="s">
         <v>243</v>
       </c>
-      <c r="F45" t="s">
-        <v>225</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>244</v>
       </c>
-      <c r="H45" t="s">
+      <c r="I45" t="s">
         <v>245</v>
       </c>
-      <c r="I45" t="s">
+      <c r="J45" t="s">
         <v>246</v>
-      </c>
-      <c r="J45" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -3079,31 +3073,31 @@
         <v>3</v>
       </c>
       <c r="B46" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C46" t="s">
+        <v>247</v>
+      </c>
+      <c r="D46" t="s">
         <v>248</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>249</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
+        <v>224</v>
+      </c>
+      <c r="G46" t="s">
         <v>250</v>
       </c>
-      <c r="F46" t="s">
-        <v>225</v>
-      </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>251</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>252</v>
       </c>
-      <c r="I46" t="s">
+      <c r="J46" t="s">
         <v>253</v>
-      </c>
-      <c r="J46" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -3111,31 +3105,31 @@
         <v>3</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C47" t="s">
+        <v>254</v>
+      </c>
+      <c r="D47" t="s">
         <v>255</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>256</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
+        <v>224</v>
+      </c>
+      <c r="G47" t="s">
         <v>257</v>
       </c>
-      <c r="F47" t="s">
-        <v>225</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>258</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
         <v>259</v>
       </c>
-      <c r="I47" t="s">
+      <c r="J47" t="s">
         <v>260</v>
-      </c>
-      <c r="J47" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -3143,31 +3137,31 @@
         <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C48" t="s">
+        <v>261</v>
+      </c>
+      <c r="D48" t="s">
         <v>262</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>263</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
+        <v>229</v>
+      </c>
+      <c r="G48" t="s">
         <v>264</v>
       </c>
-      <c r="F48" t="s">
-        <v>230</v>
-      </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>265</v>
       </c>
-      <c r="H48" t="s">
+      <c r="I48" t="s">
         <v>266</v>
       </c>
-      <c r="I48" t="s">
+      <c r="J48" t="s">
         <v>267</v>
-      </c>
-      <c r="J48" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -3175,31 +3169,31 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C49" t="s">
+        <v>268</v>
+      </c>
+      <c r="D49" t="s">
         <v>269</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>270</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49" t="s">
+        <v>229</v>
+      </c>
+      <c r="G49" t="s">
         <v>271</v>
       </c>
-      <c r="F49" t="s">
-        <v>230</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>272</v>
       </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>273</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" t="s">
         <v>274</v>
-      </c>
-      <c r="J49" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -3207,31 +3201,31 @@
         <v>3</v>
       </c>
       <c r="B50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
+        <v>275</v>
+      </c>
+      <c r="D50" t="s">
         <v>276</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>277</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
+        <v>229</v>
+      </c>
+      <c r="G50" t="s">
         <v>278</v>
       </c>
-      <c r="F50" t="s">
-        <v>230</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>279</v>
       </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
         <v>280</v>
       </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>281</v>
-      </c>
-      <c r="J50" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -3239,31 +3233,31 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" t="s">
+        <v>282</v>
+      </c>
+      <c r="D51" t="s">
         <v>283</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>284</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
+        <v>234</v>
+      </c>
+      <c r="G51" t="s">
         <v>285</v>
       </c>
-      <c r="F51" t="s">
-        <v>235</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>286</v>
       </c>
-      <c r="H51" t="s">
+      <c r="I51" t="s">
         <v>287</v>
       </c>
-      <c r="I51" t="s">
-        <v>288</v>
-      </c>
       <c r="J51" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="52" spans="1:10">
@@ -3271,31 +3265,31 @@
         <v>3</v>
       </c>
       <c r="B52" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C52" t="s">
+        <v>288</v>
+      </c>
+      <c r="D52" t="s">
         <v>289</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>290</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>234</v>
+      </c>
+      <c r="G52" t="s">
         <v>291</v>
       </c>
-      <c r="F52" t="s">
-        <v>235</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>292</v>
       </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>293</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>294</v>
-      </c>
-      <c r="J52" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="53" spans="1:10">
@@ -3303,31 +3297,31 @@
         <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C53" t="s">
+        <v>295</v>
+      </c>
+      <c r="D53" t="s">
+        <v>100</v>
+      </c>
+      <c r="E53" t="s">
+        <v>101</v>
+      </c>
+      <c r="F53" t="s">
+        <v>99</v>
+      </c>
+      <c r="G53" t="s">
         <v>296</v>
       </c>
-      <c r="D53" t="s">
-        <v>101</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="H53" t="s">
         <v>102</v>
       </c>
-      <c r="F53" t="s">
-        <v>100</v>
-      </c>
-      <c r="G53" t="s">
+      <c r="I53" t="s">
+        <v>103</v>
+      </c>
+      <c r="J53" t="s">
         <v>297</v>
-      </c>
-      <c r="H53" t="s">
-        <v>103</v>
-      </c>
-      <c r="I53" t="s">
-        <v>104</v>
-      </c>
-      <c r="J53" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -3335,31 +3329,31 @@
         <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C54" t="s">
+        <v>298</v>
+      </c>
+      <c r="D54" t="s">
         <v>299</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>300</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
+        <v>104</v>
+      </c>
+      <c r="G54" t="s">
         <v>301</v>
       </c>
-      <c r="F54" t="s">
-        <v>105</v>
-      </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>302</v>
       </c>
-      <c r="H54" t="s">
+      <c r="I54" t="s">
         <v>303</v>
       </c>
-      <c r="I54" t="s">
+      <c r="J54" t="s">
         <v>304</v>
-      </c>
-      <c r="J54" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -3367,31 +3361,31 @@
         <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C55" t="s">
+        <v>305</v>
+      </c>
+      <c r="D55" t="s">
         <v>306</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>307</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
+        <v>59</v>
+      </c>
+      <c r="G55" t="s">
         <v>308</v>
       </c>
-      <c r="F55" t="s">
-        <v>60</v>
-      </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>309</v>
       </c>
-      <c r="H55" t="s">
+      <c r="I55" t="s">
         <v>310</v>
       </c>
-      <c r="I55" t="s">
+      <c r="J55" t="s">
         <v>311</v>
-      </c>
-      <c r="J55" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -3399,31 +3393,31 @@
         <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C56" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" t="s">
         <v>313</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>314</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
+        <v>59</v>
+      </c>
+      <c r="G56" t="s">
         <v>315</v>
       </c>
-      <c r="F56" t="s">
-        <v>60</v>
-      </c>
-      <c r="G56" t="s">
+      <c r="H56" t="s">
         <v>316</v>
       </c>
-      <c r="H56" t="s">
+      <c r="I56" t="s">
         <v>317</v>
       </c>
-      <c r="I56" t="s">
+      <c r="J56" t="s">
         <v>318</v>
-      </c>
-      <c r="J56" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -3431,28 +3425,28 @@
         <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C57" t="s">
+        <v>319</v>
+      </c>
+      <c r="D57" t="s">
         <v>320</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>321</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
+        <v>186</v>
+      </c>
+      <c r="G57" t="s">
         <v>322</v>
       </c>
-      <c r="F57" t="s">
-        <v>187</v>
-      </c>
-      <c r="G57" t="s">
+      <c r="H57" t="s">
         <v>323</v>
       </c>
-      <c r="H57" t="s">
+      <c r="I57" t="s">
         <v>324</v>
-      </c>
-      <c r="I57" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -3460,31 +3454,31 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C58" t="s">
+        <v>325</v>
+      </c>
+      <c r="D58" t="s">
         <v>326</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>327</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
+        <v>186</v>
+      </c>
+      <c r="G58" t="s">
         <v>328</v>
       </c>
-      <c r="F58" t="s">
-        <v>187</v>
-      </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>329</v>
       </c>
-      <c r="H58" t="s">
+      <c r="I58" t="s">
         <v>330</v>
       </c>
-      <c r="I58" t="s">
+      <c r="J58" t="s">
         <v>331</v>
-      </c>
-      <c r="J58" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -3492,31 +3486,31 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C59" t="s">
+        <v>332</v>
+      </c>
+      <c r="D59" t="s">
         <v>333</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>334</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
+        <v>191</v>
+      </c>
+      <c r="G59" t="s">
         <v>335</v>
       </c>
-      <c r="F59" t="s">
-        <v>192</v>
-      </c>
-      <c r="G59" t="s">
+      <c r="H59" t="s">
         <v>336</v>
       </c>
-      <c r="H59" t="s">
+      <c r="I59" t="s">
         <v>337</v>
       </c>
-      <c r="I59" t="s">
+      <c r="J59" t="s">
         <v>338</v>
-      </c>
-      <c r="J59" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -3524,31 +3518,31 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C60" t="s">
+        <v>339</v>
+      </c>
+      <c r="D60" t="s">
         <v>340</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>341</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
+        <v>191</v>
+      </c>
+      <c r="G60" t="s">
         <v>342</v>
       </c>
-      <c r="F60" t="s">
-        <v>192</v>
-      </c>
-      <c r="G60" t="s">
+      <c r="H60" t="s">
         <v>343</v>
       </c>
-      <c r="H60" t="s">
+      <c r="I60" t="s">
         <v>344</v>
       </c>
-      <c r="I60" t="s">
+      <c r="J60" t="s">
         <v>345</v>
-      </c>
-      <c r="J60" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -3556,28 +3550,28 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C61" t="s">
+        <v>346</v>
+      </c>
+      <c r="D61" t="s">
+        <v>197</v>
+      </c>
+      <c r="E61" t="s">
+        <v>198</v>
+      </c>
+      <c r="F61" t="s">
+        <v>196</v>
+      </c>
+      <c r="G61" t="s">
         <v>347</v>
       </c>
-      <c r="D61" t="s">
-        <v>198</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="H61" t="s">
         <v>199</v>
       </c>
-      <c r="F61" t="s">
-        <v>197</v>
-      </c>
-      <c r="G61" t="s">
-        <v>348</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="I61" t="s">
         <v>200</v>
-      </c>
-      <c r="I61" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="62" spans="1:10">
@@ -3585,31 +3579,31 @@
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C62" t="s">
+        <v>348</v>
+      </c>
+      <c r="D62" t="s">
+        <v>202</v>
+      </c>
+      <c r="E62" t="s">
+        <v>203</v>
+      </c>
+      <c r="F62" t="s">
+        <v>201</v>
+      </c>
+      <c r="G62" t="s">
         <v>349</v>
       </c>
-      <c r="D62" t="s">
-        <v>203</v>
-      </c>
-      <c r="E62" t="s">
+      <c r="H62" t="s">
         <v>204</v>
       </c>
-      <c r="F62" t="s">
-        <v>202</v>
-      </c>
-      <c r="G62" t="s">
+      <c r="I62" t="s">
+        <v>205</v>
+      </c>
+      <c r="J62" t="s">
         <v>350</v>
-      </c>
-      <c r="H62" t="s">
-        <v>205</v>
-      </c>
-      <c r="I62" t="s">
-        <v>206</v>
-      </c>
-      <c r="J62" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -3617,31 +3611,31 @@
         <v>3</v>
       </c>
       <c r="B63" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C63" t="s">
+        <v>351</v>
+      </c>
+      <c r="D63" t="s">
+        <v>208</v>
+      </c>
+      <c r="E63" t="s">
         <v>352</v>
       </c>
-      <c r="D63" t="s">
-        <v>209</v>
-      </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
+        <v>207</v>
+      </c>
+      <c r="G63" t="s">
         <v>353</v>
       </c>
-      <c r="F63" t="s">
-        <v>208</v>
-      </c>
-      <c r="G63" t="s">
-        <v>354</v>
-      </c>
       <c r="H63" t="s">
+        <v>210</v>
+      </c>
+      <c r="I63" t="s">
         <v>211</v>
       </c>
-      <c r="I63" t="s">
+      <c r="J63" t="s">
         <v>212</v>
-      </c>
-      <c r="J63" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="64" spans="1:10">
@@ -3649,28 +3643,28 @@
         <v>3</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C64" t="s">
+        <v>354</v>
+      </c>
+      <c r="D64" t="s">
+        <v>214</v>
+      </c>
+      <c r="E64" t="s">
+        <v>215</v>
+      </c>
+      <c r="F64" t="s">
+        <v>213</v>
+      </c>
+      <c r="G64" t="s">
         <v>355</v>
       </c>
-      <c r="D64" t="s">
-        <v>215</v>
-      </c>
-      <c r="E64" t="s">
+      <c r="H64" t="s">
         <v>216</v>
       </c>
-      <c r="F64" t="s">
-        <v>214</v>
-      </c>
-      <c r="G64" t="s">
-        <v>356</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>217</v>
-      </c>
-      <c r="I64" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -3678,31 +3672,31 @@
         <v>3</v>
       </c>
       <c r="B65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C65" t="s">
+        <v>356</v>
+      </c>
+      <c r="D65" t="s">
         <v>357</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>358</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
+        <v>218</v>
+      </c>
+      <c r="G65" t="s">
         <v>359</v>
       </c>
-      <c r="F65" t="s">
-        <v>219</v>
-      </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>360</v>
       </c>
-      <c r="H65" t="s">
+      <c r="I65" t="s">
         <v>361</v>
       </c>
-      <c r="I65" t="s">
-        <v>362</v>
-      </c>
       <c r="J65" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="66" spans="1:10">
@@ -3710,31 +3704,31 @@
         <v>3</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C66" t="s">
+        <v>362</v>
+      </c>
+      <c r="D66" t="s">
         <v>363</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>364</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
+        <v>218</v>
+      </c>
+      <c r="G66" t="s">
         <v>365</v>
       </c>
-      <c r="F66" t="s">
-        <v>219</v>
-      </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>366</v>
       </c>
-      <c r="H66" t="s">
+      <c r="I66" t="s">
         <v>367</v>
       </c>
-      <c r="I66" t="s">
+      <c r="J66" t="s">
         <v>368</v>
-      </c>
-      <c r="J66" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -3742,31 +3736,31 @@
         <v>3</v>
       </c>
       <c r="B67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C67" t="s">
+        <v>369</v>
+      </c>
+      <c r="D67" t="s">
         <v>370</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>371</v>
       </c>
-      <c r="E67" t="s">
+      <c r="F67" t="s">
+        <v>104</v>
+      </c>
+      <c r="G67" t="s">
         <v>372</v>
       </c>
-      <c r="F67" t="s">
-        <v>105</v>
-      </c>
-      <c r="G67" t="s">
+      <c r="H67" t="s">
         <v>373</v>
       </c>
-      <c r="H67" t="s">
+      <c r="I67" t="s">
         <v>374</v>
       </c>
-      <c r="I67" t="s">
-        <v>375</v>
-      </c>
       <c r="J67" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -3774,28 +3768,28 @@
         <v>3</v>
       </c>
       <c r="B68" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C68" t="s">
+        <v>375</v>
+      </c>
+      <c r="D68" t="s">
         <v>376</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>377</v>
       </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
+        <v>110</v>
+      </c>
+      <c r="G68" t="s">
         <v>378</v>
       </c>
-      <c r="F68" t="s">
-        <v>111</v>
-      </c>
-      <c r="G68" t="s">
+      <c r="H68" t="s">
         <v>379</v>
       </c>
-      <c r="H68" t="s">
-        <v>380</v>
-      </c>
       <c r="I68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -3803,28 +3797,28 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C69" t="s">
+        <v>380</v>
+      </c>
+      <c r="D69" t="s">
         <v>381</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
         <v>382</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>383</v>
       </c>
-      <c r="F69" t="s">
+      <c r="G69" t="s">
         <v>384</v>
       </c>
-      <c r="G69" t="s">
+      <c r="H69" t="s">
         <v>385</v>
       </c>
-      <c r="H69" t="s">
-        <v>386</v>
-      </c>
       <c r="I69" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70" spans="1:10">
@@ -3832,28 +3826,28 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C70" t="s">
+        <v>386</v>
+      </c>
+      <c r="D70" t="s">
         <v>387</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
         <v>388</v>
       </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>389</v>
       </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>390</v>
       </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>391</v>
       </c>
-      <c r="H70" t="s">
-        <v>392</v>
-      </c>
       <c r="I70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>